<commit_message>
parser and generator changes for new format
</commit_message>
<xml_diff>
--- a/generator/diplo/sample_data_kaznu.xlsx
+++ b/generator/diplo/sample_data_kaznu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\ediploma\generator\diplo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EF85710-D07F-4B29-A34B-4CD9B4DA0015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866E1249-CFA8-4A29-8C46-12D71EE69B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -459,26 +459,26 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="5" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -769,37 +769,39 @@
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="5"/>
-    <col min="2" max="2" width="55.6640625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="21.33203125" style="5" customWidth="1"/>
-    <col min="4" max="6" width="47.6640625" style="5" customWidth="1"/>
-    <col min="7" max="8" width="36.5546875" style="5" customWidth="1"/>
-    <col min="9" max="9" width="39.6640625" style="5" customWidth="1"/>
-    <col min="10" max="10" width="37" style="5" customWidth="1"/>
-    <col min="11" max="11" width="67" style="5" customWidth="1"/>
-    <col min="12" max="12" width="24.44140625" style="5" customWidth="1"/>
-    <col min="13" max="13" width="68.6640625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="24.44140625" style="5" customWidth="1"/>
-    <col min="15" max="15" width="96.44140625" style="5" customWidth="1"/>
-    <col min="16" max="18" width="24.44140625" style="5" customWidth="1"/>
-    <col min="19" max="19" width="21.33203125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="12.44140625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="21.21875" style="1" customWidth="1"/>
-    <col min="22" max="22" width="18.44140625" style="1" customWidth="1"/>
-    <col min="23" max="23" width="19.88671875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="25.109375" style="1" customWidth="1"/>
-    <col min="25" max="25" width="25.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="36.6640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="5" customWidth="1"/>
+    <col min="4" max="5" width="38.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="15.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="39" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.5546875" style="5" customWidth="1"/>
+    <col min="13" max="13" width="44.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="39.44140625" style="5" customWidth="1"/>
+    <col min="16" max="16" width="9.5546875" style="5" customWidth="1"/>
+    <col min="17" max="17" width="7.44140625" style="5" customWidth="1"/>
+    <col min="18" max="18" width="7.33203125" style="5" customWidth="1"/>
+    <col min="19" max="19" width="50.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="28.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="25.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="12.109375" style="1" customWidth="1"/>
     <col min="27" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="16" t="s">
@@ -825,32 +827,32 @@
       </c>
       <c r="Q1" s="17"/>
       <c r="R1" s="18"/>
-      <c r="S1" s="19" t="s">
+      <c r="S1" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="T1" s="19" t="s">
+      <c r="T1" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="19" t="s">
+      <c r="U1" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="V1" s="19" t="s">
+      <c r="V1" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="W1" s="19" t="s">
+      <c r="W1" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="X1" s="19" t="s">
+      <c r="X1" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="Y1" s="19" t="s">
+      <c r="Y1" s="14" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
       <c r="D2" s="8" t="s">
         <v>6</v>
       </c>
@@ -890,13 +892,13 @@
       <c r="R2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="S2" s="20"/>
-      <c r="T2" s="20"/>
-      <c r="U2" s="20"/>
-      <c r="V2" s="20"/>
-      <c r="W2" s="20"/>
-      <c r="X2" s="20"/>
-      <c r="Y2" s="20"/>
+      <c r="S2" s="15"/>
+      <c r="T2" s="15"/>
+      <c r="U2" s="15"/>
+      <c r="V2" s="15"/>
+      <c r="W2" s="15"/>
+      <c r="X2" s="15"/>
+      <c r="Y2" s="15"/>
     </row>
     <row r="3" spans="1:25" ht="140.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
@@ -1355,6 +1357,16 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="J1:O1"/>
+    <mergeCell ref="P1:R1"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N2:O2"/>
     <mergeCell ref="X1:X2"/>
     <mergeCell ref="Y1:Y2"/>
     <mergeCell ref="S1:S2"/>
@@ -1362,16 +1374,6 @@
     <mergeCell ref="U1:U2"/>
     <mergeCell ref="V1:V2"/>
     <mergeCell ref="W1:W2"/>
-    <mergeCell ref="J1:O1"/>
-    <mergeCell ref="P1:R1"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="G1:I1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="W3" r:id="rId1" xr:uid="{72F65B7B-CC82-48B8-BBE5-661BADA831E8}"/>

</xml_diff>